<commit_message>
reports: Fix Hebrew sheet names in stops report
- 'כל התחנות' (All Stops)
- 'סיכום נהגים' (Driver Summary)
- 'סטטיסטיקה' (Statistics)

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/רשימת_תחנות_01_07_עד_05_08_26.xlsx
+++ b/reports/רשימת_תחנות_01_07_עד_05_08_26.xlsx
@@ -1,46 +1,44 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amanltd-my.sharepoint.com/personal/yuval_rasner_co_il/Documents/Claude Aman/Code/routes-report/reports/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AEADCE9-E7CF-4D63-9EA1-2179357F4F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{690B0D0B-1AB3-4527-9B7B-2234CEC80CDB}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="DailyStats" sheetId="3" r:id="rId1"/>
-    <sheet name="DriverSummary" sheetId="2" r:id="rId2"/>
-    <sheet name="AllStops" sheetId="1" r:id="rId3"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>3</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="3" baseType="lpstr">
+      <vt:lpstr>DailyStats</vt:lpstr>
+      <vt:lpstr>DriverSummary</vt:lpstr>
+      <vt:lpstr>AllStops</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Yuval Lerner</dc:creator>
+  <cp:lastModifiedBy>Yuval Lerner</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-08-06T08:11:21Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-08-06T08:11:50Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3845" uniqueCount="76">
   <si>
     <t>round</t>
@@ -273,7 +271,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -325,7 +323,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -640,7 +638,48 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amanltd-my.sharepoint.com/personal/yuval_rasner_co_il/Documents/Claude Aman/Code/routes-report/reports/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AEADCE9-E7CF-4D63-9EA1-2179357F4F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{690B0D0B-1AB3-4527-9B7B-2234CEC80CDB}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="סטטיסטיקה" sheetId="3" r:id="rId1"/>
+    <sheet name="סיכום נהגים" sheetId="2" r:id="rId2"/>
+    <sheet name="כל התחנות" sheetId="1" r:id="rId3"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C47E86D-65C8-4E52-B925-00D7BC80E527}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -649,7 +688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E7D206F-0744-41F3-9EB1-4E6DAE409399}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -658,7 +697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{572D77AF-957B-41D0-A6F6-901B34730888}">
   <dimension ref="A1:H985"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>

</xml_diff>